<commit_message>
commit de changements graphiques
</commit_message>
<xml_diff>
--- a/tabcomp (3).xlsx
+++ b/tabcomp (3).xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arthu\Documents\EPSI\RenduDocBTS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp64\www\PortfolioFin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F1EAA81-0546-481F-B326-3EA3A078E2B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{458CBB00-2C01-4E51-877C-63C2382A70D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E4" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$42</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$41</definedName>
   </definedNames>
   <calcPr calcId="101716"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -164,9 +164,6 @@
   </si>
   <si>
     <t>Création &amp; CRUD d'une base de données</t>
-  </si>
-  <si>
-    <t>Création &amp; CRUD de BDD</t>
   </si>
   <si>
     <t>SESSION 2026</t>
@@ -206,7 +203,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -281,8 +278,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="16"/>
+      <color theme="5" tint="-0.249977111117893"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -301,6 +304,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="27">
     <border>
@@ -664,7 +673,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -749,9 +758,51 @@
     <xf numFmtId="14" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -776,44 +827,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1124,7 +1139,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ88"/>
+  <dimension ref="A1:AQ87"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="70.42578125" style="1" customWidth="1"/>
@@ -1135,56 +1150,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30" t="s">
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1" s="33"/>
+    </row>
+    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="33" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+    </row>
+    <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="H1" s="30"/>
-    </row>
-    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-    </row>
-    <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="31" t="s">
-        <v>42</v>
-      </c>
-      <c r="B3" s="32"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="37" t="s">
-        <v>45</v>
-      </c>
-      <c r="G3" s="32"/>
-      <c r="H3" s="38"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="51" t="s">
+        <v>44</v>
+      </c>
+      <c r="G3" s="46"/>
+      <c r="H3" s="52"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="34" t="s">
-        <v>43</v>
-      </c>
-      <c r="B4" s="35"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="36"/>
+      <c r="A4" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="49"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="49"/>
+      <c r="E4" s="50"/>
       <c r="F4" s="7" t="s">
         <v>8</v>
       </c>
@@ -1192,27 +1207,27 @@
         <v>15</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L4" s="12"/>
     </row>
     <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="49" t="s">
-        <v>44</v>
-      </c>
-      <c r="B5" s="50"/>
-      <c r="C5" s="50"/>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="50"/>
-      <c r="G5" s="50"/>
-      <c r="H5" s="51"/>
+      <c r="A5" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="43"/>
+      <c r="C5" s="43"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="39" t="s">
+      <c r="A6" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="47" t="s">
+      <c r="B6" s="40" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="5" t="s">
@@ -1235,8 +1250,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="40"/>
-      <c r="B7" s="48"/>
+      <c r="A7" s="32"/>
+      <c r="B7" s="41"/>
       <c r="C7" s="11" t="s">
         <v>9</v>
       </c>
@@ -1292,16 +1307,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A8" s="41" t="s">
+      <c r="A8" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="42"/>
-      <c r="C8" s="42"/>
-      <c r="D8" s="42"/>
-      <c r="E8" s="42"/>
-      <c r="F8" s="42"/>
-      <c r="G8" s="42"/>
-      <c r="H8" s="43"/>
+      <c r="B8" s="35"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="35"/>
+      <c r="G8" s="35"/>
+      <c r="H8" s="36"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1397,8 +1412,8 @@
       <c r="C10" s="25"/>
       <c r="D10" s="25"/>
       <c r="E10" s="25"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="25"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="17"/>
       <c r="H10" s="26"/>
       <c r="I10"/>
       <c r="J10"/>
@@ -1446,8 +1461,8 @@
       <c r="C11" s="25"/>
       <c r="D11" s="25"/>
       <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
       <c r="H11" s="26"/>
       <c r="I11"/>
       <c r="J11"/>
@@ -1495,7 +1510,7 @@
       <c r="C12" s="25"/>
       <c r="D12" s="25"/>
       <c r="E12" s="17"/>
-      <c r="F12" s="25"/>
+      <c r="F12" s="17"/>
       <c r="G12" s="25"/>
       <c r="H12" s="26"/>
       <c r="I12"/>
@@ -1536,21 +1551,21 @@
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="20" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="B13" s="29">
-        <v>45550</v>
+        <v>45729</v>
       </c>
       <c r="C13" s="25"/>
       <c r="D13" s="17"/>
       <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
+      <c r="F13" s="25"/>
       <c r="H13" s="26"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
       <c r="L13"/>
-      <c r="M13"/>
+      <c r="M13" s="10"/>
       <c r="N13"/>
       <c r="O13"/>
       <c r="P13"/>
@@ -1584,21 +1599,22 @@
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="20" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B14" s="29">
-        <v>45729</v>
+        <v>45829</v>
       </c>
       <c r="C14" s="25"/>
       <c r="D14" s="17"/>
       <c r="E14" s="17"/>
       <c r="F14" s="25"/>
+      <c r="G14" s="17"/>
       <c r="H14" s="26"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
       <c r="L14"/>
-      <c r="M14" s="10"/>
+      <c r="M14"/>
       <c r="N14"/>
       <c r="O14"/>
       <c r="P14"/>
@@ -1632,16 +1648,16 @@
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="20" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B15" s="29">
-        <v>45829</v>
+        <v>45761</v>
       </c>
       <c r="C15" s="25"/>
-      <c r="D15" s="17"/>
+      <c r="D15" s="25"/>
       <c r="E15" s="17"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="25"/>
       <c r="H15" s="26"/>
       <c r="I15"/>
       <c r="J15"/>
@@ -1649,7 +1665,7 @@
       <c r="L15"/>
       <c r="M15"/>
       <c r="N15"/>
-      <c r="O15"/>
+      <c r="O15" s="10"/>
       <c r="P15"/>
       <c r="Q15"/>
       <c r="R15"/>
@@ -1681,16 +1697,16 @@
     </row>
     <row r="16" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="20" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B16" s="29">
-        <v>45761</v>
+        <v>46080</v>
       </c>
       <c r="C16" s="25"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="17"/>
       <c r="H16" s="26"/>
       <c r="I16"/>
       <c r="J16"/>
@@ -1698,7 +1714,7 @@
       <c r="L16"/>
       <c r="M16"/>
       <c r="N16"/>
-      <c r="O16" s="10"/>
+      <c r="O16"/>
       <c r="P16"/>
       <c r="Q16"/>
       <c r="R16"/>
@@ -1730,16 +1746,16 @@
     </row>
     <row r="17" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="20" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="B17" s="29">
-        <v>46080</v>
+        <v>46127</v>
       </c>
       <c r="C17" s="25"/>
       <c r="D17" s="17"/>
       <c r="E17" s="25"/>
       <c r="F17" s="17"/>
-      <c r="G17" s="25"/>
+      <c r="G17" s="17"/>
       <c r="H17" s="26"/>
       <c r="I17"/>
       <c r="J17"/>
@@ -1779,16 +1795,16 @@
     </row>
     <row r="18" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B18" s="29">
-        <v>46127</v>
+        <v>45990</v>
       </c>
       <c r="C18" s="25"/>
       <c r="D18" s="17"/>
       <c r="E18" s="25"/>
       <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
+      <c r="G18" s="25"/>
       <c r="H18" s="26"/>
       <c r="I18"/>
       <c r="J18"/>
@@ -1828,14 +1844,14 @@
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="20" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B19" s="29">
-        <v>45990</v>
+        <v>46102</v>
       </c>
       <c r="C19" s="25"/>
       <c r="D19" s="17"/>
-      <c r="E19" s="25"/>
+      <c r="E19" s="17"/>
       <c r="F19" s="17"/>
       <c r="G19" s="25"/>
       <c r="H19" s="26"/>
@@ -1877,14 +1893,14 @@
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="20" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="B20" s="29">
-        <v>46102</v>
+        <v>45609</v>
       </c>
       <c r="C20" s="25"/>
       <c r="D20" s="25"/>
-      <c r="E20" s="17"/>
+      <c r="E20" s="25"/>
       <c r="F20" s="17"/>
       <c r="G20" s="25"/>
       <c r="H20" s="26"/>
@@ -1926,15 +1942,15 @@
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="20" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B21" s="29">
-        <v>45609</v>
+        <v>45901</v>
       </c>
       <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
+      <c r="D21" s="17"/>
       <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
+      <c r="F21" s="25"/>
       <c r="G21" s="25"/>
       <c r="H21" s="26"/>
       <c r="I21"/>
@@ -1975,10 +1991,10 @@
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="20" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B22" s="29">
-        <v>45901</v>
+        <v>45536</v>
       </c>
       <c r="C22" s="25"/>
       <c r="D22" s="17"/>
@@ -2024,14 +2040,14 @@
     </row>
     <row r="23" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="20" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B23" s="29">
-        <v>45536</v>
+        <v>45931</v>
       </c>
       <c r="C23" s="25"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
+      <c r="D23" s="53"/>
+      <c r="E23" s="25"/>
       <c r="F23" s="17"/>
       <c r="G23" s="25"/>
       <c r="H23" s="26"/>
@@ -2073,16 +2089,16 @@
     </row>
     <row r="24" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="20" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="B24" s="29">
-        <v>45931</v>
+        <v>46332</v>
       </c>
       <c r="C24" s="25"/>
-      <c r="D24" s="25"/>
+      <c r="D24" s="17"/>
       <c r="E24" s="25"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="25"/>
+      <c r="F24" s="25"/>
+      <c r="G24" s="17"/>
       <c r="H24" s="26"/>
       <c r="I24"/>
       <c r="J24"/>
@@ -2120,19 +2136,17 @@
       <c r="AP24"/>
       <c r="AQ24"/>
     </row>
-    <row r="25" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="B25" s="29">
-        <v>46332</v>
-      </c>
-      <c r="C25" s="25"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="25"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="26"/>
+    <row r="25" spans="1:43" s="2" customFormat="1" ht="20.25" x14ac:dyDescent="0.2">
+      <c r="A25" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="B25" s="38"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="38"/>
+      <c r="H25" s="39"/>
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
@@ -2169,17 +2183,19 @@
       <c r="AP25"/>
       <c r="AQ25"/>
     </row>
-    <row r="26" spans="1:43" s="2" customFormat="1" ht="20.25" x14ac:dyDescent="0.2">
-      <c r="A26" s="44" t="s">
-        <v>19</v>
-      </c>
-      <c r="B26" s="45"/>
-      <c r="C26" s="45"/>
-      <c r="D26" s="45"/>
-      <c r="E26" s="45"/>
-      <c r="F26" s="45"/>
-      <c r="G26" s="45"/>
-      <c r="H26" s="46"/>
+    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="28">
+        <v>45769</v>
+      </c>
+      <c r="C26" s="25"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="25"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="26"/>
       <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
@@ -2218,17 +2234,17 @@
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="20" t="s">
-        <v>28</v>
-      </c>
-      <c r="B27" s="28">
+        <v>37</v>
+      </c>
+      <c r="B27" s="29">
         <v>45769</v>
       </c>
       <c r="C27" s="25"/>
       <c r="D27" s="25"/>
-      <c r="E27" s="17"/>
+      <c r="E27" s="25"/>
       <c r="F27" s="25"/>
       <c r="G27" s="25"/>
-      <c r="H27" s="26"/>
+      <c r="H27" s="25"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2266,11 +2282,11 @@
       <c r="AQ27"/>
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="20" t="s">
-        <v>37</v>
+      <c r="A28" s="23" t="s">
+        <v>38</v>
       </c>
       <c r="B28" s="29">
-        <v>45769</v>
+        <v>46134</v>
       </c>
       <c r="C28" s="25"/>
       <c r="D28" s="25"/>
@@ -2315,18 +2331,18 @@
       <c r="AQ28"/>
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="23" t="s">
-        <v>38</v>
+      <c r="A29" s="20" t="s">
+        <v>29</v>
       </c>
       <c r="B29" s="29">
         <v>46134</v>
       </c>
       <c r="C29" s="25"/>
-      <c r="D29" s="25"/>
-      <c r="E29" s="25"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
       <c r="F29" s="25"/>
-      <c r="G29" s="25"/>
-      <c r="H29" s="25"/>
+      <c r="G29" s="17"/>
+      <c r="H29" s="26"/>
       <c r="I29"/>
       <c r="J29"/>
       <c r="K29"/>
@@ -2364,18 +2380,14 @@
       <c r="AQ29"/>
     </row>
     <row r="30" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="B30" s="29">
-        <v>46134</v>
-      </c>
-      <c r="C30" s="25"/>
+      <c r="A30" s="20"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="17"/>
       <c r="D30" s="17"/>
       <c r="E30" s="17"/>
-      <c r="F30" s="25"/>
+      <c r="F30" s="17"/>
       <c r="G30" s="17"/>
-      <c r="H30" s="26"/>
+      <c r="H30" s="22"/>
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
@@ -2502,15 +2514,17 @@
       <c r="AP32"/>
       <c r="AQ32"/>
     </row>
-    <row r="33" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="20"/>
-      <c r="B33" s="21"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
-      <c r="G33" s="17"/>
-      <c r="H33" s="22"/>
+    <row r="33" spans="1:43" s="2" customFormat="1" ht="20.25" x14ac:dyDescent="0.2">
+      <c r="A33" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="B33" s="38"/>
+      <c r="C33" s="38"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="38"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="38"/>
+      <c r="H33" s="39"/>
       <c r="I33"/>
       <c r="J33"/>
       <c r="K33"/>
@@ -2547,17 +2561,19 @@
       <c r="AP33"/>
       <c r="AQ33"/>
     </row>
-    <row r="34" spans="1:43" s="2" customFormat="1" ht="20.25" x14ac:dyDescent="0.2">
-      <c r="A34" s="44" t="s">
-        <v>20</v>
-      </c>
-      <c r="B34" s="45"/>
-      <c r="C34" s="45"/>
-      <c r="D34" s="45"/>
-      <c r="E34" s="45"/>
-      <c r="F34" s="45"/>
-      <c r="G34" s="45"/>
-      <c r="H34" s="46"/>
+    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="B34" s="29">
+        <v>46041</v>
+      </c>
+      <c r="C34" s="25"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="27"/>
+      <c r="G34" s="17"/>
+      <c r="H34" s="26"/>
       <c r="I34"/>
       <c r="J34"/>
       <c r="K34"/>
@@ -2596,16 +2612,14 @@
     </row>
     <row r="35" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="B35" s="29">
-        <v>46041</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="B35" s="21"/>
       <c r="C35" s="25"/>
-      <c r="D35" s="17"/>
+      <c r="D35" s="25"/>
       <c r="E35" s="17"/>
-      <c r="F35" s="27"/>
-      <c r="G35" s="17"/>
+      <c r="F35" s="25"/>
+      <c r="G35" s="25"/>
       <c r="H35" s="26"/>
       <c r="I35"/>
       <c r="J35"/>
@@ -2645,14 +2659,14 @@
     </row>
     <row r="36" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="20" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B36" s="21"/>
       <c r="C36" s="25"/>
-      <c r="D36" s="25"/>
+      <c r="D36" s="17"/>
       <c r="E36" s="17"/>
       <c r="F36" s="25"/>
-      <c r="G36" s="25"/>
+      <c r="G36" s="17"/>
       <c r="H36" s="26"/>
       <c r="I36"/>
       <c r="J36"/>
@@ -2691,16 +2705,14 @@
       <c r="AQ36"/>
     </row>
     <row r="37" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="20" t="s">
-        <v>32</v>
-      </c>
+      <c r="A37" s="20"/>
       <c r="B37" s="21"/>
-      <c r="C37" s="25"/>
+      <c r="C37" s="17"/>
       <c r="D37" s="17"/>
       <c r="E37" s="17"/>
-      <c r="F37" s="25"/>
+      <c r="F37" s="17"/>
       <c r="G37" s="17"/>
-      <c r="H37" s="26"/>
+      <c r="H37" s="22"/>
       <c r="I37"/>
       <c r="J37"/>
       <c r="K37"/>
@@ -2783,14 +2795,14 @@
       <c r="AQ38"/>
     </row>
     <row r="39" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="20"/>
-      <c r="B39" s="21"/>
-      <c r="C39" s="17"/>
-      <c r="D39" s="17"/>
-      <c r="E39" s="17"/>
-      <c r="F39" s="17"/>
-      <c r="G39" s="17"/>
-      <c r="H39" s="22"/>
+      <c r="A39" s="14"/>
+      <c r="B39" s="15"/>
+      <c r="C39" s="16"/>
+      <c r="D39" s="16"/>
+      <c r="E39" s="16"/>
+      <c r="F39" s="16"/>
+      <c r="G39" s="16"/>
+      <c r="H39" s="18"/>
       <c r="I39"/>
       <c r="J39"/>
       <c r="K39"/>
@@ -2827,15 +2839,14 @@
       <c r="AP39"/>
       <c r="AQ39"/>
     </row>
-    <row r="40" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="14"/>
-      <c r="B40" s="15"/>
-      <c r="C40" s="16"/>
-      <c r="D40" s="16"/>
-      <c r="E40" s="16"/>
-      <c r="F40" s="16"/>
-      <c r="G40" s="16"/>
-      <c r="H40" s="18"/>
+    <row r="40" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="19"/>
+      <c r="C40" s="19"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="19"/>
+      <c r="G40" s="19"/>
+      <c r="H40" s="19"/>
       <c r="I40"/>
       <c r="J40"/>
       <c r="K40"/>
@@ -2872,14 +2883,15 @@
       <c r="AP40"/>
       <c r="AQ40"/>
     </row>
-    <row r="41" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="19"/>
-      <c r="C41" s="19"/>
-      <c r="D41" s="19"/>
-      <c r="E41" s="19"/>
-      <c r="F41" s="19"/>
-      <c r="G41" s="19"/>
-      <c r="H41" s="19"/>
+    <row r="41" spans="1:43" s="2" customFormat="1" ht="21" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="19"/>
+      <c r="B41" s="3"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="4"/>
+      <c r="H41" s="4"/>
       <c r="I41"/>
       <c r="J41"/>
       <c r="K41"/>
@@ -2916,54 +2928,10 @@
       <c r="AP41"/>
       <c r="AQ41"/>
     </row>
-    <row r="42" spans="1:43" s="2" customFormat="1" ht="21" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="19"/>
-      <c r="B42" s="3"/>
-      <c r="C42" s="4"/>
-      <c r="D42" s="4"/>
-      <c r="E42" s="4"/>
-      <c r="F42" s="4"/>
-      <c r="G42" s="4"/>
-      <c r="H42" s="4"/>
-      <c r="I42"/>
-      <c r="J42"/>
-      <c r="K42"/>
-      <c r="L42"/>
-      <c r="M42"/>
-      <c r="N42"/>
-      <c r="O42"/>
-      <c r="P42"/>
-      <c r="Q42"/>
-      <c r="R42"/>
-      <c r="S42"/>
-      <c r="T42"/>
-      <c r="U42"/>
-      <c r="V42"/>
-      <c r="W42"/>
-      <c r="X42"/>
-      <c r="Y42"/>
-      <c r="Z42"/>
-      <c r="AA42"/>
-      <c r="AB42"/>
-      <c r="AC42"/>
-      <c r="AD42"/>
-      <c r="AE42"/>
-      <c r="AF42"/>
-      <c r="AG42"/>
-      <c r="AH42"/>
-      <c r="AI42"/>
-      <c r="AJ42"/>
-      <c r="AK42"/>
-      <c r="AL42"/>
-      <c r="AM42"/>
-      <c r="AN42"/>
-      <c r="AO42"/>
-      <c r="AP42"/>
-      <c r="AQ42"/>
-    </row>
-    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="24"/>
-    </row>
+    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="24"/>
+    </row>
+    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="46" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
@@ -3008,21 +2976,20 @@
     <row r="85" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="86" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="87" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="88" customFormat="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A26:H26"/>
-    <mergeCell ref="A34:H34"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="A5:H5"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="F3:H3"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A5:H5"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>